<commit_message>
Added prometheus alerts and grafana dashboards integration
</commit_message>
<xml_diff>
--- a/Backlog/Tasks.xlsx
+++ b/Backlog/Tasks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robert\Desktop\all\Important\praca\kafka\kafka_montool\Backlog\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robert\Desktop\all\Important\praca\Materiały\kafka\kafka_montool\Backlog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32DB8DBB-E28C-451E-AB7F-6BDBC6BC91CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2AA9E0F-7B9D-4C4B-A57C-2ABDD8F6B541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="4992" windowWidth="23256" windowHeight="12456" xr2:uid="{47695776-9741-4823-B87E-216679646C64}"/>
   </bookViews>
@@ -236,7 +236,7 @@
       <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -255,6 +255,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -268,7 +274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -284,6 +290,10 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -786,27 +796,27 @@
       </c>
     </row>
     <row r="32" spans="1:2">
-      <c r="A32" t="s">
+      <c r="A32" s="8" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:1">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="7" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:1">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="7" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:1">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="7" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="36" spans="1:1">
-      <c r="A36" s="3" t="s">
+      <c r="A36" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -816,7 +826,7 @@
       </c>
     </row>
     <row r="38" spans="1:1">
-      <c r="A38" t="s">
+      <c r="A38" s="8" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>